<commit_message>
chore: run 2026-04-12 18:52 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_12_04_2026.xlsx
+++ b/logs/Consolidado_12_04_2026.xlsx
@@ -638,10 +638,10 @@
         <v>154</v>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -676,10 +676,10 @@
         <v>77</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -714,10 +714,10 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>3</v>
@@ -733,10 +733,10 @@
         <v>103</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
@@ -988,40 +988,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Antirougeurs DAY Soothing Emulsion
 Emulsão Antivermelhidão Pele Mista SPF30
 40 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/antirougeurs-day-soothing-emulsion-4878505.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>4878505</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -1068,40 +1068,40 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Antirougeurs Rosamed SPF50+
 Concentrado Hidratante Pele Tendência Vermelhidão
 30 ml</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/antirougeurs-rosamed-spf50-8429965.html</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>8429965</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -3042,40 +3042,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Dermabsolu Eco-Refill Redensifying Day Cream
 Recarga Creme anti idade Rugas e Firmeza
 50 ml</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-eco-refill-redensifying-day-cream-8152747.html</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>8152747</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -4322,40 +4322,40 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C89" s="7" t="inlineStr">
+      <c r="C89" s="5" t="inlineStr">
         <is>
           <t>MEN Shaving Gel
 Gel de Barbear Calmante sem Álcool
 150ml</t>
         </is>
       </c>
-      <c r="D89" s="7" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/men-shaving-gel-3692080.html</t>
         </is>
       </c>
-      <c r="E89" s="7" t="inlineStr"/>
-      <c r="F89" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="inlineStr">
+      <c r="E89" s="5" t="inlineStr"/>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
         <is>
           <t>3692080</t>
         </is>
       </c>
-      <c r="H89" s="7" t="inlineStr">
+      <c r="H89" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -10591,7 +10591,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>7831747</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -10719,40 +10723,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Centaury Anti-Yellowing Gray, Blond Shampoo
 Champô Centáurea BIO Neutraliza Tons Amarelos
 400 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/centaury-anti-yellowing-gray-blond-shampoo-6863851.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>6863851</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -11525,40 +11529,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Cupuaçu Reparing Very Dry Hair Shampoo
 Champô Cupuaçu BIO Repara Cabelo Muito Seco
 400 ml</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-reparing-very-dry-hair-shampoo-343983.html</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>7104602</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -11687,43 +11691,43 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>5418515</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -18569,43 +18573,43 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19365,39 +19369,39 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Protect AH Repairing Lotion After-Sun
 Leite Reparador Rosto e Corpo Pós-Solar</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-ah-repairing-lotion-after-sun-5782495.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>5782495</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19722,40 +19726,40 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Protect X-TREM Stick Invisible SPF50+
 Protetor Solar Corpo Rosto Lábios
 8 gr</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-x-trem-stick-invisible-spf50-7129109.html</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr"/>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>7129109</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="5" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -22403,40 +22407,40 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Fio Dentário Crossing Floss
 1 un</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/fio-dentario-crossing-floss-8099110.html</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr"/>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>8099110</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -25017,38 +25021,38 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
@@ -26876,38 +26880,38 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>5418515</t>
         </is>
       </c>
-      <c r="F63" s="7" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>

</xml_diff>